<commit_message>
Respaldo de sesión completa antes de force-push de limpieza de historial
Snapshot de todo el trabajo de esta sesión (seguridad multi-tenant, migración
de anexos a Supabase Storage, motor Viabilidad IA v3.0, unificación de UI,
páginas legales, rotación de JWT_SECRET) preservado en esta rama antes de
purgar el historial de git (que contenía JWT_SECRET filtrado en 2 commits
antiguos) y hacer force-push a origin/main.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FOTOS PROY3/comunicacion mutua.xlsx
+++ b/FOTOS PROY3/comunicacion mutua.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\2026 AI EGIOC5\Antigravity JS\proyectos\Proy_03_RadarFondos\FOTOS PROY3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E105CD1-99B2-4A65-B126-342276554774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43C2E674-E792-4C0C-B685-96F998AC3C62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D643C3F9-6D41-4651-9F32-197106AA3439}"/>
   </bookViews>
@@ -536,7 +536,13 @@
       <alignment horizontal="left" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -557,13 +563,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -892,1007 +892,927 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="15"/>
-      <c r="O1" s="15"/>
-      <c r="P1" s="15"/>
-      <c r="Q1" s="15"/>
-      <c r="R1" s="15"/>
-      <c r="S1" s="15"/>
-      <c r="T1" s="16"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
+      <c r="R1" s="8"/>
+      <c r="S1" s="8"/>
+      <c r="T1" s="9"/>
     </row>
     <row r="2" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="8" t="s">
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="8" t="s">
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
-      <c r="N2" s="9"/>
-      <c r="O2" s="10"/>
-      <c r="P2" s="8" t="s">
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="Q2" s="9"/>
-      <c r="R2" s="9"/>
-      <c r="S2" s="9"/>
-      <c r="T2" s="10"/>
+      <c r="Q2" s="11"/>
+      <c r="R2" s="11"/>
+      <c r="S2" s="11"/>
+      <c r="T2" s="12"/>
     </row>
     <row r="3" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="8" t="s">
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="8" t="s">
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="8" t="s">
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="11"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="Q3" s="9"/>
-      <c r="R3" s="9"/>
-      <c r="S3" s="9"/>
-      <c r="T3" s="10"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="11"/>
+      <c r="S3" s="11"/>
+      <c r="T3" s="12"/>
     </row>
     <row r="4" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="8" t="s">
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="8" t="s">
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="10"/>
-      <c r="P4" s="8" t="s">
+      <c r="L4" s="11"/>
+      <c r="M4" s="11"/>
+      <c r="N4" s="11"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="Q4" s="9"/>
-      <c r="R4" s="9"/>
-      <c r="S4" s="9"/>
-      <c r="T4" s="10"/>
+      <c r="Q4" s="11"/>
+      <c r="R4" s="11"/>
+      <c r="S4" s="11"/>
+      <c r="T4" s="12"/>
     </row>
     <row r="5" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="8" t="s">
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="8" t="s">
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
-      <c r="N5" s="9"/>
-      <c r="O5" s="10"/>
-      <c r="P5" s="8" t="s">
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+      <c r="N5" s="11"/>
+      <c r="O5" s="12"/>
+      <c r="P5" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="Q5" s="9"/>
-      <c r="R5" s="9"/>
-      <c r="S5" s="9"/>
-      <c r="T5" s="10"/>
+      <c r="Q5" s="11"/>
+      <c r="R5" s="11"/>
+      <c r="S5" s="11"/>
+      <c r="T5" s="12"/>
     </row>
     <row r="6" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12"/>
-      <c r="N6" s="12"/>
-      <c r="O6" s="12"/>
-      <c r="P6" s="12"/>
-      <c r="Q6" s="12"/>
-      <c r="R6" s="12"/>
-      <c r="S6" s="12"/>
-      <c r="T6" s="13"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="14"/>
+      <c r="P6" s="14"/>
+      <c r="Q6" s="14"/>
+      <c r="R6" s="14"/>
+      <c r="S6" s="14"/>
+      <c r="T6" s="15"/>
     </row>
     <row r="7" spans="1:20" s="1" customFormat="1" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-      <c r="P7" s="7"/>
-      <c r="Q7" s="7"/>
-      <c r="R7" s="7"/>
-      <c r="S7" s="7"/>
-      <c r="T7" s="7"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="16"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="16"/>
+      <c r="S7" s="16"/>
+      <c r="T7" s="16"/>
     </row>
     <row r="8" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="15"/>
-      <c r="M8" s="15"/>
-      <c r="N8" s="15"/>
-      <c r="O8" s="15"/>
-      <c r="P8" s="15"/>
-      <c r="Q8" s="15"/>
-      <c r="R8" s="15"/>
-      <c r="S8" s="15"/>
-      <c r="T8" s="16"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="8"/>
+      <c r="T8" s="9"/>
     </row>
     <row r="9" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="8" t="s">
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="8" t="s">
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="8" t="s">
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="10"/>
-      <c r="Q9" s="8" t="s">
+      <c r="N9" s="11"/>
+      <c r="O9" s="11"/>
+      <c r="P9" s="12"/>
+      <c r="Q9" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="R9" s="9"/>
-      <c r="S9" s="9"/>
-      <c r="T9" s="10"/>
+      <c r="R9" s="11"/>
+      <c r="S9" s="11"/>
+      <c r="T9" s="12"/>
     </row>
     <row r="10" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="8" t="s">
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="8" t="s">
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="8" t="s">
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="12"/>
+      <c r="M10" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="N10" s="9"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="10"/>
-      <c r="Q10" s="8" t="s">
+      <c r="N10" s="11"/>
+      <c r="O10" s="11"/>
+      <c r="P10" s="12"/>
+      <c r="Q10" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="R10" s="9"/>
-      <c r="S10" s="9"/>
-      <c r="T10" s="10"/>
+      <c r="R10" s="11"/>
+      <c r="S10" s="11"/>
+      <c r="T10" s="12"/>
     </row>
     <row r="11" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="8" t="s">
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="8" t="s">
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="8" t="s">
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="N11" s="9"/>
-      <c r="O11" s="9"/>
-      <c r="P11" s="10"/>
-      <c r="Q11" s="8" t="s">
+      <c r="N11" s="11"/>
+      <c r="O11" s="11"/>
+      <c r="P11" s="12"/>
+      <c r="Q11" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="R11" s="9"/>
-      <c r="S11" s="9"/>
-      <c r="T11" s="10"/>
+      <c r="R11" s="11"/>
+      <c r="S11" s="11"/>
+      <c r="T11" s="12"/>
     </row>
     <row r="12" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="8" t="s">
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="8" t="s">
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="10"/>
-      <c r="M12" s="8" t="s">
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="12"/>
+      <c r="M12" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="N12" s="9"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="10"/>
-      <c r="Q12" s="8" t="s">
+      <c r="N12" s="11"/>
+      <c r="O12" s="11"/>
+      <c r="P12" s="12"/>
+      <c r="Q12" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="R12" s="9"/>
-      <c r="S12" s="9"/>
-      <c r="T12" s="10"/>
+      <c r="R12" s="11"/>
+      <c r="S12" s="11"/>
+      <c r="T12" s="12"/>
     </row>
     <row r="13" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="12"/>
-      <c r="N13" s="12"/>
-      <c r="O13" s="12"/>
-      <c r="P13" s="12"/>
-      <c r="Q13" s="12"/>
-      <c r="R13" s="12"/>
-      <c r="S13" s="12"/>
-      <c r="T13" s="13"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="14"/>
+      <c r="K13" s="14"/>
+      <c r="L13" s="14"/>
+      <c r="M13" s="14"/>
+      <c r="N13" s="14"/>
+      <c r="O13" s="14"/>
+      <c r="P13" s="14"/>
+      <c r="Q13" s="14"/>
+      <c r="R13" s="14"/>
+      <c r="S13" s="14"/>
+      <c r="T13" s="15"/>
     </row>
     <row r="14" spans="1:20" s="1" customFormat="1" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-      <c r="L14" s="7"/>
-      <c r="M14" s="7"/>
-      <c r="N14" s="7"/>
-      <c r="O14" s="7"/>
-      <c r="P14" s="7"/>
-      <c r="Q14" s="7"/>
-      <c r="R14" s="7"/>
-      <c r="S14" s="7"/>
-      <c r="T14" s="7"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="16"/>
+      <c r="M14" s="16"/>
+      <c r="N14" s="16"/>
+      <c r="O14" s="16"/>
+      <c r="P14" s="16"/>
+      <c r="Q14" s="16"/>
+      <c r="R14" s="16"/>
+      <c r="S14" s="16"/>
+      <c r="T14" s="16"/>
     </row>
     <row r="15" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="15"/>
-      <c r="L15" s="15"/>
-      <c r="M15" s="15"/>
-      <c r="N15" s="15"/>
-      <c r="O15" s="15"/>
-      <c r="P15" s="15"/>
-      <c r="Q15" s="15"/>
-      <c r="R15" s="15"/>
-      <c r="S15" s="15"/>
-      <c r="T15" s="16"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="8"/>
+      <c r="R15" s="8"/>
+      <c r="S15" s="8"/>
+      <c r="T15" s="9"/>
     </row>
     <row r="16" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="8" t="s">
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="8" t="s">
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
-      <c r="L16" s="10"/>
-      <c r="M16" s="8" t="s">
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="12"/>
+      <c r="M16" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="N16" s="9"/>
-      <c r="O16" s="9"/>
-      <c r="P16" s="10"/>
-      <c r="Q16" s="8" t="s">
+      <c r="N16" s="11"/>
+      <c r="O16" s="11"/>
+      <c r="P16" s="12"/>
+      <c r="Q16" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="R16" s="9"/>
-      <c r="S16" s="9"/>
-      <c r="T16" s="10"/>
+      <c r="R16" s="11"/>
+      <c r="S16" s="11"/>
+      <c r="T16" s="12"/>
     </row>
     <row r="17" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="8" t="s">
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="8" t="s">
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="J17" s="9"/>
-      <c r="K17" s="9"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="8" t="s">
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="N17" s="9"/>
-      <c r="O17" s="9"/>
-      <c r="P17" s="10"/>
-      <c r="Q17" s="8" t="s">
+      <c r="N17" s="11"/>
+      <c r="O17" s="11"/>
+      <c r="P17" s="12"/>
+      <c r="Q17" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="R17" s="9"/>
-      <c r="S17" s="9"/>
-      <c r="T17" s="10"/>
+      <c r="R17" s="11"/>
+      <c r="S17" s="11"/>
+      <c r="T17" s="12"/>
     </row>
     <row r="18" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="8" t="s">
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="8" t="s">
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="J18" s="9"/>
-      <c r="K18" s="9"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="8" t="s">
+      <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="N18" s="9"/>
-      <c r="O18" s="9"/>
-      <c r="P18" s="10"/>
-      <c r="Q18" s="8" t="s">
+      <c r="N18" s="11"/>
+      <c r="O18" s="11"/>
+      <c r="P18" s="12"/>
+      <c r="Q18" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="R18" s="9"/>
-      <c r="S18" s="9"/>
-      <c r="T18" s="10"/>
+      <c r="R18" s="11"/>
+      <c r="S18" s="11"/>
+      <c r="T18" s="12"/>
     </row>
     <row r="19" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="8" t="s">
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="8" t="s">
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="J19" s="9"/>
-      <c r="K19" s="9"/>
-      <c r="L19" s="10"/>
-      <c r="M19" s="8" t="s">
+      <c r="J19" s="11"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="N19" s="9"/>
-      <c r="O19" s="9"/>
-      <c r="P19" s="10"/>
-      <c r="Q19" s="8" t="s">
+      <c r="N19" s="11"/>
+      <c r="O19" s="11"/>
+      <c r="P19" s="12"/>
+      <c r="Q19" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="R19" s="9"/>
-      <c r="S19" s="9"/>
-      <c r="T19" s="10"/>
+      <c r="R19" s="11"/>
+      <c r="S19" s="11"/>
+      <c r="T19" s="12"/>
     </row>
     <row r="20" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
-      <c r="L20" s="12"/>
-      <c r="M20" s="12"/>
-      <c r="N20" s="12"/>
-      <c r="O20" s="12"/>
-      <c r="P20" s="12"/>
-      <c r="Q20" s="12"/>
-      <c r="R20" s="12"/>
-      <c r="S20" s="12"/>
-      <c r="T20" s="13"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="14"/>
+      <c r="K20" s="14"/>
+      <c r="L20" s="14"/>
+      <c r="M20" s="14"/>
+      <c r="N20" s="14"/>
+      <c r="O20" s="14"/>
+      <c r="P20" s="14"/>
+      <c r="Q20" s="14"/>
+      <c r="R20" s="14"/>
+      <c r="S20" s="14"/>
+      <c r="T20" s="15"/>
     </row>
     <row r="21" spans="1:20" s="1" customFormat="1" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7"/>
-      <c r="M21" s="7"/>
-      <c r="N21" s="7"/>
-      <c r="O21" s="7"/>
-      <c r="P21" s="7"/>
-      <c r="Q21" s="7"/>
-      <c r="R21" s="7"/>
-      <c r="S21" s="7"/>
-      <c r="T21" s="7"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="16"/>
+      <c r="N21" s="16"/>
+      <c r="O21" s="16"/>
+      <c r="P21" s="16"/>
+      <c r="Q21" s="16"/>
+      <c r="R21" s="16"/>
+      <c r="S21" s="16"/>
+      <c r="T21" s="16"/>
     </row>
     <row r="22" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15"/>
-      <c r="L22" s="15"/>
-      <c r="M22" s="15"/>
-      <c r="N22" s="15"/>
-      <c r="O22" s="15"/>
-      <c r="P22" s="15"/>
-      <c r="Q22" s="15"/>
-      <c r="R22" s="15"/>
-      <c r="S22" s="15"/>
-      <c r="T22" s="16"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
+      <c r="O22" s="8"/>
+      <c r="P22" s="8"/>
+      <c r="Q22" s="8"/>
+      <c r="R22" s="8"/>
+      <c r="S22" s="8"/>
+      <c r="T22" s="9"/>
     </row>
     <row r="23" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="8" t="s">
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="8" t="s">
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="L23" s="9"/>
-      <c r="M23" s="9"/>
-      <c r="N23" s="9"/>
-      <c r="O23" s="10"/>
-      <c r="P23" s="8" t="s">
+      <c r="L23" s="11"/>
+      <c r="M23" s="11"/>
+      <c r="N23" s="11"/>
+      <c r="O23" s="12"/>
+      <c r="P23" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="Q23" s="9"/>
-      <c r="R23" s="9"/>
-      <c r="S23" s="9"/>
-      <c r="T23" s="10"/>
+      <c r="Q23" s="11"/>
+      <c r="R23" s="11"/>
+      <c r="S23" s="11"/>
+      <c r="T23" s="12"/>
     </row>
     <row r="24" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="8" t="s">
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="10"/>
-      <c r="K24" s="8" t="s">
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L24" s="9"/>
-      <c r="M24" s="9"/>
-      <c r="N24" s="9"/>
-      <c r="O24" s="10"/>
-      <c r="P24" s="8" t="s">
+      <c r="L24" s="11"/>
+      <c r="M24" s="11"/>
+      <c r="N24" s="11"/>
+      <c r="O24" s="12"/>
+      <c r="P24" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="Q24" s="9"/>
-      <c r="R24" s="9"/>
-      <c r="S24" s="9"/>
-      <c r="T24" s="10"/>
+      <c r="Q24" s="11"/>
+      <c r="R24" s="11"/>
+      <c r="S24" s="11"/>
+      <c r="T24" s="12"/>
     </row>
     <row r="25" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="8" t="s">
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="10"/>
-      <c r="K25" s="8" t="s">
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="L25" s="9"/>
-      <c r="M25" s="9"/>
-      <c r="N25" s="9"/>
-      <c r="O25" s="10"/>
-      <c r="P25" s="8" t="s">
+      <c r="L25" s="11"/>
+      <c r="M25" s="11"/>
+      <c r="N25" s="11"/>
+      <c r="O25" s="12"/>
+      <c r="P25" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="Q25" s="9"/>
-      <c r="R25" s="9"/>
-      <c r="S25" s="9"/>
-      <c r="T25" s="10"/>
+      <c r="Q25" s="11"/>
+      <c r="R25" s="11"/>
+      <c r="S25" s="11"/>
+      <c r="T25" s="12"/>
     </row>
     <row r="26" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="8" t="s">
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="8" t="s">
+      <c r="G26" s="11"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="L26" s="9"/>
-      <c r="M26" s="9"/>
-      <c r="N26" s="9"/>
-      <c r="O26" s="10"/>
-      <c r="P26" s="8" t="s">
+      <c r="L26" s="11"/>
+      <c r="M26" s="11"/>
+      <c r="N26" s="11"/>
+      <c r="O26" s="12"/>
+      <c r="P26" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="Q26" s="9"/>
-      <c r="R26" s="9"/>
-      <c r="S26" s="9"/>
-      <c r="T26" s="10"/>
+      <c r="Q26" s="11"/>
+      <c r="R26" s="11"/>
+      <c r="S26" s="11"/>
+      <c r="T26" s="12"/>
     </row>
     <row r="27" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="12"/>
-      <c r="I27" s="12"/>
-      <c r="J27" s="12"/>
-      <c r="K27" s="12"/>
-      <c r="L27" s="12"/>
-      <c r="M27" s="12"/>
-      <c r="N27" s="12"/>
-      <c r="O27" s="12"/>
-      <c r="P27" s="12"/>
-      <c r="Q27" s="12"/>
-      <c r="R27" s="12"/>
-      <c r="S27" s="12"/>
-      <c r="T27" s="13"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
+      <c r="I27" s="14"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="14"/>
+      <c r="L27" s="14"/>
+      <c r="M27" s="14"/>
+      <c r="N27" s="14"/>
+      <c r="O27" s="14"/>
+      <c r="P27" s="14"/>
+      <c r="Q27" s="14"/>
+      <c r="R27" s="14"/>
+      <c r="S27" s="14"/>
+      <c r="T27" s="15"/>
     </row>
     <row r="28" spans="1:20" s="1" customFormat="1" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="7"/>
-      <c r="J28" s="7"/>
-      <c r="K28" s="7"/>
-      <c r="L28" s="7"/>
-      <c r="M28" s="7"/>
-      <c r="N28" s="7"/>
-      <c r="O28" s="7"/>
-      <c r="P28" s="7"/>
-      <c r="Q28" s="7"/>
-      <c r="R28" s="7"/>
-      <c r="S28" s="7"/>
-      <c r="T28" s="7"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="16"/>
+      <c r="I28" s="16"/>
+      <c r="J28" s="16"/>
+      <c r="K28" s="16"/>
+      <c r="L28" s="16"/>
+      <c r="M28" s="16"/>
+      <c r="N28" s="16"/>
+      <c r="O28" s="16"/>
+      <c r="P28" s="16"/>
+      <c r="Q28" s="16"/>
+      <c r="R28" s="16"/>
+      <c r="S28" s="16"/>
+      <c r="T28" s="16"/>
     </row>
     <row r="29" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B29" s="15"/>
-      <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="15"/>
-      <c r="F29" s="15"/>
-      <c r="G29" s="15"/>
-      <c r="H29" s="15"/>
-      <c r="I29" s="15"/>
-      <c r="J29" s="15"/>
-      <c r="K29" s="15"/>
-      <c r="L29" s="15"/>
-      <c r="M29" s="15"/>
-      <c r="N29" s="15"/>
-      <c r="O29" s="15"/>
-      <c r="P29" s="15"/>
-      <c r="Q29" s="15"/>
-      <c r="R29" s="15"/>
-      <c r="S29" s="15"/>
-      <c r="T29" s="16"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="8"/>
+      <c r="M29" s="8"/>
+      <c r="N29" s="8"/>
+      <c r="O29" s="8"/>
+      <c r="P29" s="8"/>
+      <c r="Q29" s="8"/>
+      <c r="R29" s="8"/>
+      <c r="S29" s="8"/>
+      <c r="T29" s="9"/>
     </row>
     <row r="30" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="8" t="s">
+      <c r="A30" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="8" t="s">
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
-      <c r="I30" s="9"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="8" t="s">
+      <c r="G30" s="11"/>
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="L30" s="9"/>
-      <c r="M30" s="9"/>
-      <c r="N30" s="9"/>
-      <c r="O30" s="10"/>
-      <c r="P30" s="8" t="s">
+      <c r="L30" s="11"/>
+      <c r="M30" s="11"/>
+      <c r="N30" s="11"/>
+      <c r="O30" s="12"/>
+      <c r="P30" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="Q30" s="9"/>
-      <c r="R30" s="9"/>
-      <c r="S30" s="9"/>
-      <c r="T30" s="10"/>
+      <c r="Q30" s="11"/>
+      <c r="R30" s="11"/>
+      <c r="S30" s="11"/>
+      <c r="T30" s="12"/>
     </row>
     <row r="31" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B31" s="9"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="8" t="s">
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="G31" s="9"/>
-      <c r="H31" s="9"/>
-      <c r="I31" s="9"/>
-      <c r="J31" s="10"/>
-      <c r="K31" s="8" t="s">
+      <c r="G31" s="11"/>
+      <c r="H31" s="11"/>
+      <c r="I31" s="11"/>
+      <c r="J31" s="12"/>
+      <c r="K31" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="L31" s="9"/>
-      <c r="M31" s="9"/>
-      <c r="N31" s="9"/>
-      <c r="O31" s="10"/>
-      <c r="P31" s="8" t="s">
+      <c r="L31" s="11"/>
+      <c r="M31" s="11"/>
+      <c r="N31" s="11"/>
+      <c r="O31" s="12"/>
+      <c r="P31" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="Q31" s="9"/>
-      <c r="R31" s="9"/>
-      <c r="S31" s="9"/>
-      <c r="T31" s="10"/>
+      <c r="Q31" s="11"/>
+      <c r="R31" s="11"/>
+      <c r="S31" s="11"/>
+      <c r="T31" s="12"/>
     </row>
     <row r="32" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="8" t="s">
+      <c r="A32" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="B32" s="9"/>
-      <c r="C32" s="9"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="8" t="s">
+      <c r="B32" s="11"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="G32" s="9"/>
-      <c r="H32" s="9"/>
-      <c r="I32" s="9"/>
-      <c r="J32" s="10"/>
-      <c r="K32" s="8" t="s">
+      <c r="G32" s="11"/>
+      <c r="H32" s="11"/>
+      <c r="I32" s="11"/>
+      <c r="J32" s="12"/>
+      <c r="K32" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="L32" s="9"/>
-      <c r="M32" s="9"/>
-      <c r="N32" s="9"/>
-      <c r="O32" s="10"/>
-      <c r="P32" s="8" t="s">
+      <c r="L32" s="11"/>
+      <c r="M32" s="11"/>
+      <c r="N32" s="11"/>
+      <c r="O32" s="12"/>
+      <c r="P32" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="Q32" s="9"/>
-      <c r="R32" s="9"/>
-      <c r="S32" s="9"/>
-      <c r="T32" s="10"/>
+      <c r="Q32" s="11"/>
+      <c r="R32" s="11"/>
+      <c r="S32" s="11"/>
+      <c r="T32" s="12"/>
     </row>
     <row r="33" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="8" t="s">
+      <c r="A33" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="B33" s="9"/>
-      <c r="C33" s="9"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="8" t="s">
+      <c r="B33" s="11"/>
+      <c r="C33" s="11"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="G33" s="9"/>
-      <c r="H33" s="9"/>
-      <c r="I33" s="9"/>
-      <c r="J33" s="10"/>
-      <c r="K33" s="8" t="s">
+      <c r="G33" s="11"/>
+      <c r="H33" s="11"/>
+      <c r="I33" s="11"/>
+      <c r="J33" s="12"/>
+      <c r="K33" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="L33" s="9"/>
-      <c r="M33" s="9"/>
-      <c r="N33" s="9"/>
-      <c r="O33" s="10"/>
-      <c r="P33" s="8" t="s">
+      <c r="L33" s="11"/>
+      <c r="M33" s="11"/>
+      <c r="N33" s="11"/>
+      <c r="O33" s="12"/>
+      <c r="P33" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="Q33" s="9"/>
-      <c r="R33" s="9"/>
-      <c r="S33" s="9"/>
-      <c r="T33" s="10"/>
+      <c r="Q33" s="11"/>
+      <c r="R33" s="11"/>
+      <c r="S33" s="11"/>
+      <c r="T33" s="12"/>
     </row>
     <row r="34" spans="1:20" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="11" t="s">
+      <c r="A34" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="B34" s="12"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="12"/>
-      <c r="I34" s="12"/>
-      <c r="J34" s="12"/>
-      <c r="K34" s="12"/>
-      <c r="L34" s="12"/>
-      <c r="M34" s="12"/>
-      <c r="N34" s="12"/>
-      <c r="O34" s="12"/>
-      <c r="P34" s="12"/>
-      <c r="Q34" s="12"/>
-      <c r="R34" s="12"/>
-      <c r="S34" s="12"/>
-      <c r="T34" s="13"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+      <c r="I34" s="14"/>
+      <c r="J34" s="14"/>
+      <c r="K34" s="14"/>
+      <c r="L34" s="14"/>
+      <c r="M34" s="14"/>
+      <c r="N34" s="14"/>
+      <c r="O34" s="14"/>
+      <c r="P34" s="14"/>
+      <c r="Q34" s="14"/>
+      <c r="R34" s="14"/>
+      <c r="S34" s="14"/>
+      <c r="T34" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="102">
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="F2:J2"/>
-    <mergeCell ref="K2:O2"/>
-    <mergeCell ref="P2:T2"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="F5:J5"/>
-    <mergeCell ref="K5:O5"/>
-    <mergeCell ref="P5:T5"/>
-    <mergeCell ref="A6:T6"/>
-    <mergeCell ref="A8:T8"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="F3:J3"/>
-    <mergeCell ref="K3:O3"/>
-    <mergeCell ref="P3:T3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:J4"/>
-    <mergeCell ref="K4:O4"/>
-    <mergeCell ref="P4:T4"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="E9:H9"/>
-    <mergeCell ref="I9:L9"/>
-    <mergeCell ref="M9:P9"/>
-    <mergeCell ref="Q9:T9"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="E10:H10"/>
-    <mergeCell ref="I10:L10"/>
-    <mergeCell ref="M10:P10"/>
-    <mergeCell ref="Q10:T10"/>
-    <mergeCell ref="A13:T13"/>
-    <mergeCell ref="A15:T15"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="E16:H16"/>
-    <mergeCell ref="I16:L16"/>
-    <mergeCell ref="M16:P16"/>
-    <mergeCell ref="Q16:T16"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="E11:H11"/>
-    <mergeCell ref="I11:L11"/>
-    <mergeCell ref="M11:P11"/>
-    <mergeCell ref="Q11:T11"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="E12:H12"/>
-    <mergeCell ref="I12:L12"/>
-    <mergeCell ref="M12:P12"/>
-    <mergeCell ref="Q12:T12"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="E19:H19"/>
-    <mergeCell ref="I19:L19"/>
-    <mergeCell ref="M19:P19"/>
-    <mergeCell ref="Q19:T19"/>
-    <mergeCell ref="A20:T20"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="E17:H17"/>
-    <mergeCell ref="I17:L17"/>
-    <mergeCell ref="M17:P17"/>
-    <mergeCell ref="Q17:T17"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="E18:H18"/>
-    <mergeCell ref="I18:L18"/>
-    <mergeCell ref="M18:P18"/>
-    <mergeCell ref="Q18:T18"/>
-    <mergeCell ref="F25:J25"/>
-    <mergeCell ref="K25:O25"/>
-    <mergeCell ref="P25:T25"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="F26:J26"/>
-    <mergeCell ref="K26:O26"/>
-    <mergeCell ref="P26:T26"/>
-    <mergeCell ref="A22:T22"/>
-    <mergeCell ref="A23:E23"/>
-    <mergeCell ref="F23:J23"/>
-    <mergeCell ref="K23:O23"/>
-    <mergeCell ref="P23:T23"/>
-    <mergeCell ref="A24:E24"/>
-    <mergeCell ref="F24:J24"/>
-    <mergeCell ref="K24:O24"/>
-    <mergeCell ref="P24:T24"/>
-    <mergeCell ref="G7:T7"/>
-    <mergeCell ref="G14:T14"/>
     <mergeCell ref="G21:T21"/>
     <mergeCell ref="G28:T28"/>
     <mergeCell ref="A33:E33"/>
@@ -1915,6 +1835,86 @@
     <mergeCell ref="K30:O30"/>
     <mergeCell ref="P30:T30"/>
     <mergeCell ref="A25:E25"/>
+    <mergeCell ref="F25:J25"/>
+    <mergeCell ref="K25:O25"/>
+    <mergeCell ref="P25:T25"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="F26:J26"/>
+    <mergeCell ref="K26:O26"/>
+    <mergeCell ref="P26:T26"/>
+    <mergeCell ref="A22:T22"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="F23:J23"/>
+    <mergeCell ref="K23:O23"/>
+    <mergeCell ref="P23:T23"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="F24:J24"/>
+    <mergeCell ref="K24:O24"/>
+    <mergeCell ref="P24:T24"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="E19:H19"/>
+    <mergeCell ref="I19:L19"/>
+    <mergeCell ref="M19:P19"/>
+    <mergeCell ref="Q19:T19"/>
+    <mergeCell ref="A20:T20"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="E17:H17"/>
+    <mergeCell ref="I17:L17"/>
+    <mergeCell ref="M17:P17"/>
+    <mergeCell ref="Q17:T17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="E18:H18"/>
+    <mergeCell ref="I18:L18"/>
+    <mergeCell ref="M18:P18"/>
+    <mergeCell ref="Q18:T18"/>
+    <mergeCell ref="A13:T13"/>
+    <mergeCell ref="A15:T15"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="E16:H16"/>
+    <mergeCell ref="I16:L16"/>
+    <mergeCell ref="M16:P16"/>
+    <mergeCell ref="Q16:T16"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="E11:H11"/>
+    <mergeCell ref="I11:L11"/>
+    <mergeCell ref="M11:P11"/>
+    <mergeCell ref="Q11:T11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="E12:H12"/>
+    <mergeCell ref="I12:L12"/>
+    <mergeCell ref="M12:P12"/>
+    <mergeCell ref="Q12:T12"/>
+    <mergeCell ref="G14:T14"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="I9:L9"/>
+    <mergeCell ref="M9:P9"/>
+    <mergeCell ref="Q9:T9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="E10:H10"/>
+    <mergeCell ref="I10:L10"/>
+    <mergeCell ref="M10:P10"/>
+    <mergeCell ref="Q10:T10"/>
+    <mergeCell ref="A6:T6"/>
+    <mergeCell ref="A8:T8"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="F3:J3"/>
+    <mergeCell ref="K3:O3"/>
+    <mergeCell ref="P3:T3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:J4"/>
+    <mergeCell ref="K4:O4"/>
+    <mergeCell ref="P4:T4"/>
+    <mergeCell ref="G7:T7"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="K2:O2"/>
+    <mergeCell ref="P2:T2"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="F5:J5"/>
+    <mergeCell ref="K5:O5"/>
+    <mergeCell ref="P5:T5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>